<commit_message>
feat: improve invoice import/manual entry and fix client selection bug
</commit_message>
<xml_diff>
--- a/test-data/payment_orders.xlsx
+++ b/test-data/payment_orders.xlsx
@@ -404,16 +404,16 @@
         <v>Fecha</v>
       </c>
       <c r="B1" t="str">
-        <v>Número</v>
+        <v>Número de OP</v>
       </c>
       <c r="C1" t="str">
-        <v>Entidad (Nombre o CUIT)</v>
+        <v>Proveedor (Nombre o CUIT)</v>
       </c>
       <c r="D1" t="str">
         <v>Monto Total</v>
       </c>
       <c r="E1" t="str">
-        <v>Medio</v>
+        <v>Medio de Pago</v>
       </c>
       <c r="F1" t="str">
         <v>Banco</v>

</xml_diff>